<commit_message>
Added Jupyter example script
</commit_message>
<xml_diff>
--- a/sample_data/sample_cell_model.xlsx
+++ b/sample_data/sample_cell_model.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomasdolezal/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomasdolezal/Documents/Baterky/TestProfiles/Python_modules_3_1/sample_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758AD7B7-55A8-7048-979D-691FB9FB5931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E9D7237-FDBC-4F40-9E8D-73BD036C85F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -190,7 +190,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -209,6 +209,13 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -279,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -291,7 +298,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -723,18 +731,18 @@
       <c r="D10" s="3"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="8">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="A12" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="8">
         <v>21</v>
       </c>
     </row>

</xml_diff>